<commit_message>
some outdoor plants added
</commit_message>
<xml_diff>
--- a/data/Outdoor plants.xlsx
+++ b/data/Outdoor plants.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BE3DB1-27BA-4371-BA64-E2E38D7641AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864A14B6-36A8-4AC0-AEDC-E5B1A128FA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8B519764-563C-4CD5-B8E9-9B8B0702B21B}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1572" uniqueCount="546">
   <si>
     <t>Plant ID</t>
   </si>
@@ -1385,13 +1385,307 @@
   </si>
   <si>
     <t>https://i.postimg.cc/HxtvL89W/spathodea-campanulata.jpg</t>
+  </si>
+  <si>
+    <t>Cycas revoluta</t>
+  </si>
+  <si>
+    <t>OP-053</t>
+  </si>
+  <si>
+    <t>سيكاس</t>
+  </si>
+  <si>
+    <t>Palms</t>
+  </si>
+  <si>
+    <t>Ficus (Bonsai)</t>
+  </si>
+  <si>
+    <t>فيكس بونساي</t>
+  </si>
+  <si>
+    <t>Ficus lyrata</t>
+  </si>
+  <si>
+    <t>فيكس ليراتا (تينة الكمان)</t>
+  </si>
+  <si>
+    <t>Strelitzia nicolai</t>
+  </si>
+  <si>
+    <t>نجمة الطيور العملاقة</t>
+  </si>
+  <si>
+    <t>فيكس ميكروكاربا</t>
+  </si>
+  <si>
+    <t>زنبق الكانا</t>
+  </si>
+  <si>
+    <t>800 - 1200</t>
+  </si>
+  <si>
+    <t>1100 - 1600</t>
+  </si>
+  <si>
+    <t>Zamia furfuracea</t>
+  </si>
+  <si>
+    <t>زاميا (نخيل الكرتون)</t>
+  </si>
+  <si>
+    <t>Ficus elastica</t>
+  </si>
+  <si>
+    <t>شجرة المطاط</t>
+  </si>
+  <si>
+    <t>OP-054</t>
+  </si>
+  <si>
+    <t>OP-055</t>
+  </si>
+  <si>
+    <t>OP-056</t>
+  </si>
+  <si>
+    <t>OP-057</t>
+  </si>
+  <si>
+    <t>OP-058</t>
+  </si>
+  <si>
+    <t>OP-059</t>
+  </si>
+  <si>
+    <t>OP-060</t>
+  </si>
+  <si>
+    <t>1 - 3 m</t>
+  </si>
+  <si>
+    <t>0.3 - 1 m</t>
+  </si>
+  <si>
+    <t>3 - 12 m</t>
+  </si>
+  <si>
+    <t>6 - 8 m</t>
+  </si>
+  <si>
+    <t>0.6 - 2.4 m</t>
+  </si>
+  <si>
+    <t>3 - 10 m</t>
+  </si>
+  <si>
+    <t>1.5 - 3 m</t>
+  </si>
+  <si>
+    <t>2 - 3.5 m</t>
+  </si>
+  <si>
+    <t>1.5 - 2 m</t>
+  </si>
+  <si>
+    <t>2 - 5 m</t>
+  </si>
+  <si>
+    <t>800-1000 g/year</t>
+  </si>
+  <si>
+    <t>300-500 g/year</t>
+  </si>
+  <si>
+    <t>1500-2000 g/year</t>
+  </si>
+  <si>
+    <t>1800-2500 g/year</t>
+  </si>
+  <si>
+    <t>1800-2200 g/year</t>
+  </si>
+  <si>
+    <t>800-1200 g/year</t>
+  </si>
+  <si>
+    <t>600-900 g/year</t>
+  </si>
+  <si>
+    <t>1600-2100 g/year</t>
+  </si>
+  <si>
+    <t>1100-1300 g/year</t>
+  </si>
+  <si>
+    <t>400-600 g/year</t>
+  </si>
+  <si>
+    <t>2000-3000 g/year</t>
+  </si>
+  <si>
+    <t>2500-3500 g/year</t>
+  </si>
+  <si>
+    <t>2500-3000 g/year</t>
+  </si>
+  <si>
+    <t>1100-1600 g/year</t>
+  </si>
+  <si>
+    <t>800-1100 g/year</t>
+  </si>
+  <si>
+    <t>2200-2800 g/year</t>
+  </si>
+  <si>
+    <t>Ficus microcarpa (panda)</t>
+  </si>
+  <si>
+    <t>Canna generalis</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/wT8pc3Nj/Cycas-revoluta.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/5NdVqjz4/Canna-generalis.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/kX3mFDS5/Ficus-(Bonsai).jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/5NdVqjz0/Ficus-elastica.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/Nfqc7LXX/Ficus-lyrata.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/pXbHYyjz/Ficus-microcarpa-(panda).jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/28RDF3WQ/Strelitzia-nicolai.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/SNFh7j9d/Zamia-furfuracea.jpg</t>
+  </si>
+  <si>
+    <t>Plectranthus amboinicus</t>
+  </si>
+  <si>
+    <t>الفوطن</t>
+  </si>
+  <si>
+    <t>400 - 650</t>
+  </si>
+  <si>
+    <t>Pelargonium graveolens</t>
+  </si>
+  <si>
+    <t>العطرة</t>
+  </si>
+  <si>
+    <t>550 - 800</t>
+  </si>
+  <si>
+    <t>Rosmarinus officinalis</t>
+  </si>
+  <si>
+    <t>روز ماري</t>
+  </si>
+  <si>
+    <t>500 - 750</t>
+  </si>
+  <si>
+    <t>700 - 1000</t>
+  </si>
+  <si>
+    <t>Cymbopogon citratus</t>
+  </si>
+  <si>
+    <t>عشب الليمون</t>
+  </si>
+  <si>
+    <t>Lavandula angustifolia</t>
+  </si>
+  <si>
+    <t>لافندر</t>
+  </si>
+  <si>
+    <t>550 - 850</t>
+  </si>
+  <si>
+    <t>Salvia officinalis</t>
+  </si>
+  <si>
+    <t>مرامية</t>
+  </si>
+  <si>
+    <t>Myrtus communis</t>
+  </si>
+  <si>
+    <t>حنا الياس</t>
+  </si>
+  <si>
+    <t>OP-061</t>
+  </si>
+  <si>
+    <t>OP-062</t>
+  </si>
+  <si>
+    <t>OP-063</t>
+  </si>
+  <si>
+    <t>OP-064</t>
+  </si>
+  <si>
+    <t>OP-065</t>
+  </si>
+  <si>
+    <t>OP-066</t>
+  </si>
+  <si>
+    <t>OP-067</t>
+  </si>
+  <si>
+    <t>0.5 - 1.5 m</t>
+  </si>
+  <si>
+    <t>500-750 g/year</t>
+  </si>
+  <si>
+    <t>400-650 g/year</t>
+  </si>
+  <si>
+    <t>350-550 g/year</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/L8njHStr/Cymbopogon-citratus.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/kXjx3GSr/Lavandula-angustifolia.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/SNZWFRMB/Myrtus-communis.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/Qx6pGCTv/Pelargonium-graveolens.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/X72wSq5n/Plectranthus-amboinicus.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/3JLg5NGY/Rosmarinus-officinalis.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/ZKfrtnNb/Salvia-officinalis.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1450,6 +1744,16 @@
       <name val="Calibri"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1459,12 +1763,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1473,7 +1792,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1532,8 +1851,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1899,7 +2227,7 @@
     <col min="2" max="2" width="32.453125" style="4" customWidth="1"/>
     <col min="3" max="3" width="23.1796875" style="4" customWidth="1"/>
     <col min="4" max="4" width="12.453125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="47.81640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="54.453125" style="4" customWidth="1"/>
     <col min="6" max="6" width="17.7265625" style="4" customWidth="1"/>
     <col min="7" max="7" width="15.26953125" style="4" customWidth="1"/>
     <col min="8" max="8" width="16.81640625" style="4" bestFit="1" customWidth="1"/>
@@ -5461,91 +5789,1066 @@
       <c r="B53" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="C53" s="28" t="s">
+      <c r="C53" s="25" t="s">
         <v>442</v>
       </c>
       <c r="E53" s="12" t="s">
         <v>447</v>
       </c>
-      <c r="F53" s="28" t="s">
+      <c r="F53" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="G53" s="28" t="s">
+      <c r="G53" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="H53" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="I53" s="28" t="s">
+      <c r="H53" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="I53" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="J53" s="28" t="s">
+      <c r="J53" s="25" t="s">
         <v>443</v>
       </c>
-      <c r="K53" s="28" t="s">
+      <c r="K53" s="25" t="s">
         <v>444</v>
       </c>
-      <c r="L53" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="M53" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="N53" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="O53" s="28" t="s">
+      <c r="L53" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="M53" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="N53" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="O53" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="P53" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q53" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="R53" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="S53" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="T53" s="28" t="s">
+      <c r="P53" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q53" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="R53" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="S53" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="T53" s="25" t="s">
         <v>445</v>
       </c>
-      <c r="U53" s="28" t="s">
+      <c r="U53" s="25" t="s">
         <v>446</v>
       </c>
-      <c r="V53" s="28" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="54" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="55" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="56" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="57" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="58" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="59" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="60" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="61" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="62" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="63" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="64" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="65" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="66" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="67" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="68" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="69" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="70" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="71" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="72" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="73" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="74" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="75" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="76" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="77" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="78" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="79" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="80" ht="14.5" x14ac:dyDescent="0.35"/>
+      <c r="V53" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A54" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="B54" s="29" t="s">
+        <v>448</v>
+      </c>
+      <c r="C54" s="28" t="s">
+        <v>450</v>
+      </c>
+      <c r="D54" s="30"/>
+      <c r="E54" s="31" t="s">
+        <v>501</v>
+      </c>
+      <c r="F54" s="29" t="s">
+        <v>451</v>
+      </c>
+      <c r="G54" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H54" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I54" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="J54" s="29" t="s">
+        <v>473</v>
+      </c>
+      <c r="K54" s="29" t="s">
+        <v>473</v>
+      </c>
+      <c r="L54" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M54" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N54" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="O54" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="P54" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q54" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R54" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S54" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T54" s="29" t="s">
+        <v>483</v>
+      </c>
+      <c r="U54" s="29" t="s">
+        <v>491</v>
+      </c>
+      <c r="V54" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A55" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="B55" s="29" t="s">
+        <v>452</v>
+      </c>
+      <c r="C55" s="28" t="s">
+        <v>453</v>
+      </c>
+      <c r="D55" s="30"/>
+      <c r="E55" s="31" t="s">
+        <v>503</v>
+      </c>
+      <c r="F55" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G55" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H55" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I55" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="J55" s="29" t="s">
+        <v>474</v>
+      </c>
+      <c r="K55" s="29" t="s">
+        <v>474</v>
+      </c>
+      <c r="L55" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M55" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N55" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="O55" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P55" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q55" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="R55" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S55" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T55" s="29" t="s">
+        <v>484</v>
+      </c>
+      <c r="U55" s="29" t="s">
+        <v>492</v>
+      </c>
+      <c r="V55" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A56" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="B56" s="29" t="s">
+        <v>454</v>
+      </c>
+      <c r="C56" s="28" t="s">
+        <v>455</v>
+      </c>
+      <c r="D56" s="30"/>
+      <c r="E56" s="31" t="s">
+        <v>505</v>
+      </c>
+      <c r="F56" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="G56" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H56" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I56" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="J56" s="29" t="s">
+        <v>475</v>
+      </c>
+      <c r="K56" s="29" t="s">
+        <v>479</v>
+      </c>
+      <c r="L56" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M56" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N56" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O56" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P56" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q56" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="R56" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S56" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="T56" s="29" t="s">
+        <v>485</v>
+      </c>
+      <c r="U56" s="29" t="s">
+        <v>493</v>
+      </c>
+      <c r="V56" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A57" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B57" s="29" t="s">
+        <v>456</v>
+      </c>
+      <c r="C57" s="28" t="s">
+        <v>457</v>
+      </c>
+      <c r="D57" s="30"/>
+      <c r="E57" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="F57" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G57" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H57" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I57" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J57" s="29" t="s">
+        <v>476</v>
+      </c>
+      <c r="K57" s="29" t="s">
+        <v>480</v>
+      </c>
+      <c r="L57" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M57" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N57" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O57" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P57" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q57" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R57" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S57" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="T57" s="29" t="s">
+        <v>486</v>
+      </c>
+      <c r="U57" s="29" t="s">
+        <v>494</v>
+      </c>
+      <c r="V57" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A58" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="B58" s="29" t="s">
+        <v>499</v>
+      </c>
+      <c r="C58" s="28" t="s">
+        <v>458</v>
+      </c>
+      <c r="D58" s="30"/>
+      <c r="E58" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="F58" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="G58" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H58" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I58" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J58" s="29" t="s">
+        <v>358</v>
+      </c>
+      <c r="K58" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="L58" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="M58" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N58" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O58" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="P58" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q58" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R58" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S58" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="T58" s="29" t="s">
+        <v>487</v>
+      </c>
+      <c r="U58" s="29" t="s">
+        <v>495</v>
+      </c>
+      <c r="V58" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A59" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="B59" s="29" t="s">
+        <v>500</v>
+      </c>
+      <c r="C59" s="28" t="s">
+        <v>459</v>
+      </c>
+      <c r="D59" s="30"/>
+      <c r="E59" s="31" t="s">
+        <v>502</v>
+      </c>
+      <c r="F59" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G59" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H59" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I59" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J59" s="29" t="s">
+        <v>477</v>
+      </c>
+      <c r="K59" s="29" t="s">
+        <v>474</v>
+      </c>
+      <c r="L59" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M59" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="N59" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O59" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P59" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q59" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R59" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S59" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T59" s="29" t="s">
+        <v>488</v>
+      </c>
+      <c r="U59" s="29" t="s">
+        <v>496</v>
+      </c>
+      <c r="V59" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A60" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="B60" s="29" t="s">
+        <v>462</v>
+      </c>
+      <c r="C60" s="28" t="s">
+        <v>463</v>
+      </c>
+      <c r="D60" s="30"/>
+      <c r="E60" s="31" t="s">
+        <v>508</v>
+      </c>
+      <c r="F60" s="29" t="s">
+        <v>451</v>
+      </c>
+      <c r="G60" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H60" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I60" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="J60" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="K60" s="29" t="s">
+        <v>481</v>
+      </c>
+      <c r="L60" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M60" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N60" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="O60" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="P60" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q60" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R60" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S60" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T60" s="29" t="s">
+        <v>489</v>
+      </c>
+      <c r="U60" s="29" t="s">
+        <v>497</v>
+      </c>
+      <c r="V60" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A61" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B61" s="29" t="s">
+        <v>464</v>
+      </c>
+      <c r="C61" s="28" t="s">
+        <v>465</v>
+      </c>
+      <c r="D61" s="30"/>
+      <c r="E61" s="31" t="s">
+        <v>504</v>
+      </c>
+      <c r="F61" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="G61" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H61" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I61" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="J61" s="29" t="s">
+        <v>478</v>
+      </c>
+      <c r="K61" s="29" t="s">
+        <v>482</v>
+      </c>
+      <c r="L61" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M61" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N61" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O61" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="P61" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q61" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R61" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S61" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="T61" s="29" t="s">
+        <v>490</v>
+      </c>
+      <c r="U61" s="29" t="s">
+        <v>498</v>
+      </c>
+      <c r="V61" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="B62" s="29" t="s">
+        <v>509</v>
+      </c>
+      <c r="C62" s="28" t="s">
+        <v>510</v>
+      </c>
+      <c r="D62" s="30"/>
+      <c r="E62" s="31" t="s">
+        <v>543</v>
+      </c>
+      <c r="F62" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G62" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H62" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I62" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="J62" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="K62" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="L62" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M62" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N62" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="O62" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P62" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q62" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R62" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S62" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T62" s="29" t="s">
+        <v>484</v>
+      </c>
+      <c r="U62" s="29" t="s">
+        <v>511</v>
+      </c>
+      <c r="V62" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A63" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B63" s="29" t="s">
+        <v>512</v>
+      </c>
+      <c r="C63" s="28" t="s">
+        <v>513</v>
+      </c>
+      <c r="D63" s="30"/>
+      <c r="E63" s="31" t="s">
+        <v>542</v>
+      </c>
+      <c r="F63" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G63" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H63" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I63" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J63" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="K63" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="L63" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M63" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N63" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O63" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P63" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q63" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R63" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S63" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T63" s="29" t="s">
+        <v>492</v>
+      </c>
+      <c r="U63" s="29" t="s">
+        <v>514</v>
+      </c>
+      <c r="V63" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A64" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B64" s="29" t="s">
+        <v>515</v>
+      </c>
+      <c r="C64" s="28" t="s">
+        <v>516</v>
+      </c>
+      <c r="D64" s="30"/>
+      <c r="E64" s="31" t="s">
+        <v>544</v>
+      </c>
+      <c r="F64" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G64" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H64" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I64" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J64" s="29" t="s">
+        <v>535</v>
+      </c>
+      <c r="K64" s="29" t="s">
+        <v>535</v>
+      </c>
+      <c r="L64" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M64" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N64" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O64" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P64" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q64" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R64" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S64" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T64" s="29" t="s">
+        <v>536</v>
+      </c>
+      <c r="U64" s="29" t="s">
+        <v>518</v>
+      </c>
+      <c r="V64" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="65" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A65" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="B65" s="29" t="s">
+        <v>519</v>
+      </c>
+      <c r="C65" s="28" t="s">
+        <v>520</v>
+      </c>
+      <c r="D65" s="30"/>
+      <c r="E65" s="31" t="s">
+        <v>539</v>
+      </c>
+      <c r="F65" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="G65" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H65" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I65" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J65" s="29" t="s">
+        <v>354</v>
+      </c>
+      <c r="K65" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="L65" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M65" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N65" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O65" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P65" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q65" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R65" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="S65" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T65" s="29" t="s">
+        <v>489</v>
+      </c>
+      <c r="U65" s="29" t="s">
+        <v>460</v>
+      </c>
+      <c r="V65" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A66" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="B66" s="29" t="s">
+        <v>521</v>
+      </c>
+      <c r="C66" s="28" t="s">
+        <v>522</v>
+      </c>
+      <c r="D66" s="30"/>
+      <c r="E66" s="31" t="s">
+        <v>540</v>
+      </c>
+      <c r="F66" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G66" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H66" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I66" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J66" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="K66" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="L66" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M66" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N66" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O66" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P66" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q66" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R66" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S66" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T66" s="29" t="s">
+        <v>537</v>
+      </c>
+      <c r="U66" s="29" t="s">
+        <v>523</v>
+      </c>
+      <c r="V66" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A67" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="B67" s="29" t="s">
+        <v>524</v>
+      </c>
+      <c r="C67" s="28" t="s">
+        <v>525</v>
+      </c>
+      <c r="D67" s="30"/>
+      <c r="E67" s="31" t="s">
+        <v>545</v>
+      </c>
+      <c r="F67" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G67" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H67" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I67" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J67" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="K67" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="L67" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M67" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N67" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O67" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P67" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q67" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R67" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S67" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="T67" s="29" t="s">
+        <v>538</v>
+      </c>
+      <c r="U67" s="29" t="s">
+        <v>517</v>
+      </c>
+      <c r="V67" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="68" spans="1:22" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A68" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="B68" s="29" t="s">
+        <v>526</v>
+      </c>
+      <c r="C68" s="28" t="s">
+        <v>527</v>
+      </c>
+      <c r="D68" s="30"/>
+      <c r="E68" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="F68" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G68" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H68" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I68" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="J68" s="29" t="s">
+        <v>482</v>
+      </c>
+      <c r="K68" s="29" t="s">
+        <v>479</v>
+      </c>
+      <c r="L68" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="M68" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N68" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="O68" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="P68" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q68" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="R68" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S68" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="T68" s="29" t="s">
+        <v>488</v>
+      </c>
+      <c r="U68" s="29" t="s">
+        <v>461</v>
+      </c>
+      <c r="V68" s="25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="69" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="70" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="71" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="72" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="73" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="74" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="75" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="76" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="77" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="78" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="79" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="80" spans="1:22" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="81" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="82" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="83" ht="14.5" x14ac:dyDescent="0.35"/>
@@ -5647,11 +6950,11 @@
     <sortCondition ref="A2:A37"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="B51:B52">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B53:B1048576 B46:B50 B37:B38 B20:B35 B1:B14">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B51:B52">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
   <dataValidations count="8">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1" xr:uid="{58D66573-3890-4498-A66F-3227660DC8D7}"/>
@@ -5782,6 +7085,21 @@
     <hyperlink ref="E6" r:id="rId102" xr:uid="{38F1636E-04EF-45FA-A853-30396B0673BC}"/>
     <hyperlink ref="D6" r:id="rId103" xr:uid="{C2587916-F827-41B7-8EDB-D66AF039E12E}"/>
     <hyperlink ref="E53" r:id="rId104" xr:uid="{10833195-DF06-4765-8492-81FB0535DD3A}"/>
+    <hyperlink ref="E54" r:id="rId105" xr:uid="{6B6B6FD5-94FB-4C3F-8C6D-C8F98D39BF55}"/>
+    <hyperlink ref="E59" r:id="rId106" xr:uid="{7A2F8379-D88C-42CF-9E91-A348C4939CD0}"/>
+    <hyperlink ref="E55" r:id="rId107" xr:uid="{17ABCE55-2212-4EAC-9742-C819791C2C70}"/>
+    <hyperlink ref="E61" r:id="rId108" xr:uid="{CF8803C5-144C-4D5F-82DF-F61B938CA47D}"/>
+    <hyperlink ref="E56" r:id="rId109" xr:uid="{1C667421-4AFB-434D-B095-36B1E491B074}"/>
+    <hyperlink ref="E58" r:id="rId110" xr:uid="{0BCCC82D-074A-459C-B18D-9FB4BA4D2B9D}"/>
+    <hyperlink ref="E57" r:id="rId111" xr:uid="{6E2163E2-0911-46D1-9A34-538BC6563894}"/>
+    <hyperlink ref="E60" r:id="rId112" xr:uid="{3E86BEB0-40CE-4260-AC99-EB7BFFB0D05E}"/>
+    <hyperlink ref="E65" r:id="rId113" xr:uid="{F42A429F-D5AD-425E-9219-A70672FE74D5}"/>
+    <hyperlink ref="E66" r:id="rId114" xr:uid="{9DF583C0-6C0B-44DF-8A1F-E70EEC85103F}"/>
+    <hyperlink ref="E68" r:id="rId115" xr:uid="{D7B14A4B-6E71-4186-9719-F317C904BDF8}"/>
+    <hyperlink ref="E63" r:id="rId116" xr:uid="{8756E56E-041E-4F59-9969-C5616368EFD9}"/>
+    <hyperlink ref="E62" r:id="rId117" xr:uid="{B1D664C3-3084-49EE-88BA-925083CE2BB4}"/>
+    <hyperlink ref="E64" r:id="rId118" xr:uid="{26EB60D1-3355-4405-BD5C-5F387663B5A5}"/>
+    <hyperlink ref="E67" r:id="rId119" xr:uid="{8688C54A-1F4E-4850-B6DD-9DA6D3EEA4C5}"/>
   </hyperlinks>
   <printOptions verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6707,15 +8025,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000D89A625C5B6364BB7302BED22ED65DA" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="05bac8ad6e033965382d52c38353e541">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7855343b-5261-4afc-a17c-d4c130fbaa85" xmlns:ns4="72f917e0-5d36-43ac-975d-26afa4cf7fc0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="452e5605b09f318b6d66379e79837bd5" ns3:_="" ns4:_="">
     <xsd:import namespace="7855343b-5261-4afc-a17c-d4c130fbaa85"/>
@@ -6962,6 +8271,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6971,14 +8289,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BE4A15A-EC2D-4537-B6DC-2F235DBE6314}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56978299-3DC6-451D-A1E5-57FB07C431CC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6997,6 +8307,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BE4A15A-EC2D-4537-B6DC-2F235DBE6314}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F53F9CFB-0E7D-4BF1-9CBE-0D133C6536E4}">
   <ds:schemaRefs>

</xml_diff>